<commit_message>
Record the live Vercel deployment in the tracker and checkpoint form
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pyu1PuNoiQSXEChGBbiq3J
</commit_message>
<xml_diff>
--- a/project-docs/phase-3/tracker/Group Y - ITC327W Phase 3 Project Progress Tracker (updated 20 Oct).xlsx
+++ b/project-docs/phase-3/tracker/Group Y - ITC327W Phase 3 Project Progress Tracker (updated 20 Oct).xlsx
@@ -716,7 +716,7 @@
       </x:c>
       <x:c r="E5" s="46" t="n">
         <x:f>COUNTIF('Development Progress'!G4:G33,"Completed")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -729,7 +729,7 @@
       </x:c>
       <x:c r="E6" s="46" t="n">
         <x:f>COUNTIF('Development Progress'!G4:G33,"In Progress")</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -759,7 +759,7 @@
       </x:c>
       <x:c r="E8" s="47" t="n">
         <x:f>IFERROR(AVERAGE('Development Progress'!H4:H33),0)</x:f>
-        <x:v>0.46199999999999997</x:v>
+        <x:v>0.474</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1516,18 +1516,20 @@
       <x:c r="E24" s="34" t="str">
         <x:v>2026-10-20</x:v>
       </x:c>
-      <x:c r="F24" s="34"/>
+      <x:c r="F24" s="34" t="str">
+        <x:v>2026-10-20</x:v>
+      </x:c>
       <x:c r="G24" s="34" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H24" s="54" t="n">
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I24" s="34" t="str">
         <x:v>web/Dockerfile.vercel; project-docs/phase-3/hosting-on-vercel.md</x:v>
       </x:c>
       <x:c r="J24" s="34" t="str">
-        <x:v>Project and Dockerfile ready; web app runs against the live Supabase project (checked locally 20 Oct). Supabase settings could not be added from the assistant (no access to the Vercel team); add them in the Vercel dashboard, then deploy.</x:v>
+        <x:v>Live at https://riese-auto-clinic.vercel.app (20 Oct). Checked: login as mechanic and admin, dashboard, booking page, /Track; WhatsApp message links to /Track; mechanic sees no finalize/delete, admin does.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2026,21 +2028,35 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="34" t="str"/>
-      <x:c r="B10" s="34" t="str"/>
-      <x:c r="C10" s="34" t="str"/>
-      <x:c r="D10" s="34" t="str"/>
-      <x:c r="E10" s="34" t="str"/>
-      <x:c r="F10" s="34" t="str"/>
+      <x:c r="A10" s="34" t="str">
+        <x:v>Wisani Nkuna</x:v>
+      </x:c>
+      <x:c r="B10" s="34" t="str">
+        <x:v>222010787</x:v>
+      </x:c>
+      <x:c r="C10" s="34" t="str">
+        <x:v>ASP.NET</x:v>
+      </x:c>
+      <x:c r="D10" s="34" t="str">
+        <x:v>Hosting</x:v>
+      </x:c>
+      <x:c r="E10" s="34" t="str">
+        <x:v>Web app deployed on Vercel; fixed the login HTTP 400 (shared encryption key across containers); checked the live site with both staff accounts</x:v>
+      </x:c>
+      <x:c r="F10" s="34" t="str">
+        <x:v>2026-10-20</x:v>
+      </x:c>
       <x:c r="G10" s="34" t="str"/>
-      <x:c r="H10" s="34" t="str"/>
+      <x:c r="H10" s="34" t="str">
+        <x:v>web/Auth/FixedKeyRepository.cs; https://riese-auto-clinic.vercel.app</x:v>
+      </x:c>
       <x:c r="I10" s="34" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="J10" s="34" t="str"/>
       <x:c r="K10" s="34" t="str"/>
       <x:c r="L10" s="34" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -4236,17 +4252,33 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="34" t="str"/>
-      <x:c r="B19" s="34" t="str"/>
-      <x:c r="C19" s="34" t="str"/>
-      <x:c r="D19" s="34" t="str"/>
-      <x:c r="E19" s="34" t="str"/>
-      <x:c r="F19" s="34" t="str"/>
+      <x:c r="A19" s="34" t="str">
+        <x:v>2026-10-20</x:v>
+      </x:c>
+      <x:c r="B19" s="34" t="str">
+        <x:v>Login failed with HTTP 400 on Vercel</x:v>
+      </x:c>
+      <x:c r="C19" s="34" t="str">
+        <x:v>Staff could not log in reliably; would also cause random logouts</x:v>
+      </x:c>
+      <x:c r="D19" s="34" t="str">
+        <x:v>Every container now uses the same encryption key from the DataProtection__Secret setting (web/Auth/FixedKeyRepository.cs)</x:v>
+      </x:c>
+      <x:c r="E19" s="34" t="str">
+        <x:v>Wisani Nkuna</x:v>
+      </x:c>
+      <x:c r="F19" s="34" t="str">
+        <x:v>2026-10-20</x:v>
+      </x:c>
       <x:c r="G19" s="34" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="H19" s="34" t="str"/>
-      <x:c r="I19" s="34" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="H19" s="34" t="str">
+        <x:v>2026-10-20</x:v>
+      </x:c>
+      <x:c r="I19" s="34" t="str">
+        <x:v>Reproduced and fixed locally, then confirmed on the live site.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="34" t="str"/>
@@ -4508,7 +4540,7 @@
         <x:v>What was completed during Phase 3?</x:v>
       </x:c>
       <x:c r="B5" s="34" t="str">
-        <x:v>Both apps already run on one shared Supabase project with the main functions built (Phases 1-2). Since 15 Oct: Send on WhatsApp in the web app, Riese titles for Google, migrations 0010 and 0011, web app prepared for Vercel, Unit 4 readiness pack mapping every function and shared process.</x:v>
+        <x:v>Both apps already run on one shared Supabase project with the main functions built (Phases 1-2). Since 15 Oct: Send on WhatsApp in the web app, Riese titles for Google, migrations 0010 and 0011, web app prepared for Vercel, Unit 4 readiness pack mapping every function and shared process. 20 Oct: web app live on Vercel (riese-auto-clinic.vercel.app), checked with both staff accounts.</x:v>
       </x:c>
       <x:c r="C5" s="34"/>
       <x:c r="E5" t="str">
@@ -4523,7 +4555,7 @@
         <x:v>Which functions or processes remain incomplete?</x:v>
       </x:c>
       <x:c r="B6" s="34" t="str">
-        <x:v>Migrations 0009/0004/0010/0011 to run on the live project (0008 is live); Flutter WhatsApp button, pull-to-refresh, add part through add_booking_part and web build; one labour ledger; web admin role from profiles; logged-in evidence and the P1/P2 recording; SRS implementation section; MS Project; web app deployed on Vercel.</x:v>
+        <x:v>Migrations 0009/0004/0010/0011 to run on the live project (0008 is live); Flutter WhatsApp button, pull-to-refresh, add part through add_booking_part and web build; one labour ledger; web admin role from profiles; logged-in evidence and the P1/P2 recording; SRS implementation section; MS Project.</x:v>
       </x:c>
       <x:c r="C6" s="34"/>
       <x:c r="E6" t="str">

</xml_diff>